<commit_message>
Force dark theme configuration
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aeiou\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aeiou\Constructor_Academy\Streamlit_Inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{55115599-59E7-4878-AA2A-DA5271F25D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB22309-C071-47D0-AEA0-3705E7D87546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{FCD79D1D-7458-46B7-8965-31719ED767EB}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="269">
   <si>
     <t>dr_code</t>
   </si>
@@ -585,15 +585,9 @@
     <t>BG</t>
   </si>
   <si>
-    <t>H</t>
-  </si>
-  <si>
     <t>AW</t>
   </si>
   <si>
-    <t>I</t>
-  </si>
-  <si>
     <t>AX</t>
   </si>
   <si>
@@ -829,6 +823,18 @@
   </si>
   <si>
     <t>ET</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>BH</t>
+  </si>
+  <si>
+    <t>BI</t>
+  </si>
+  <si>
+    <t>T</t>
   </si>
 </sst>
 </file>
@@ -1741,10 +1747,10 @@
         <v>144</v>
       </c>
       <c r="C3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E3" t="s">
         <v>143</v>
@@ -1758,10 +1764,10 @@
         <v>145</v>
       </c>
       <c r="C4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E4" t="s">
         <v>143</v>
@@ -1775,10 +1781,10 @@
         <v>146</v>
       </c>
       <c r="C5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E5" t="s">
         <v>143</v>
@@ -1792,10 +1798,10 @@
         <v>147</v>
       </c>
       <c r="C6" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E6" t="s">
         <v>143</v>
@@ -1809,10 +1815,10 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E7" t="s">
         <v>143</v>
@@ -1826,10 +1832,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E8" t="s">
         <v>143</v>
@@ -1979,10 +1985,10 @@
         <v>156</v>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E17" t="s">
         <v>143</v>
@@ -2948,10 +2954,10 @@
         <v>46</v>
       </c>
       <c r="C74" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D74" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E74" t="s">
         <v>143</v>
@@ -2965,10 +2971,10 @@
         <v>47</v>
       </c>
       <c r="C75" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D75" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E75" t="s">
         <v>143</v>
@@ -2982,10 +2988,10 @@
         <v>48</v>
       </c>
       <c r="C76" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D76" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E76" t="s">
         <v>143</v>
@@ -2999,10 +3005,10 @@
         <v>49</v>
       </c>
       <c r="C77" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D77" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E77" t="s">
         <v>143</v>
@@ -3016,10 +3022,10 @@
         <v>50</v>
       </c>
       <c r="C78" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D78" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E78" t="s">
         <v>143</v>
@@ -3033,10 +3039,10 @@
         <v>51</v>
       </c>
       <c r="C79" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D79" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E79" t="s">
         <v>143</v>
@@ -3050,10 +3056,10 @@
         <v>52</v>
       </c>
       <c r="C80" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D80" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E80" t="s">
         <v>143</v>
@@ -3067,10 +3073,10 @@
         <v>53</v>
       </c>
       <c r="C81" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D81" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E81" t="s">
         <v>143</v>
@@ -3118,10 +3124,10 @@
         <v>56</v>
       </c>
       <c r="C84" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D84" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E84" t="s">
         <v>143</v>
@@ -3135,10 +3141,10 @@
         <v>57</v>
       </c>
       <c r="C85" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D85" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E85" t="s">
         <v>143</v>
@@ -3475,10 +3481,10 @@
         <v>77</v>
       </c>
       <c r="C105" t="s">
+        <v>241</v>
+      </c>
+      <c r="D105" t="s">
         <v>243</v>
-      </c>
-      <c r="D105" t="s">
-        <v>245</v>
       </c>
       <c r="E105" t="s">
         <v>143</v>
@@ -3492,10 +3498,10 @@
         <v>78</v>
       </c>
       <c r="C106" t="s">
+        <v>242</v>
+      </c>
+      <c r="D106" t="s">
         <v>244</v>
-      </c>
-      <c r="D106" t="s">
-        <v>246</v>
       </c>
       <c r="E106" t="s">
         <v>143</v>
@@ -3662,10 +3668,10 @@
         <v>86</v>
       </c>
       <c r="C116" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D116" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E116" t="s">
         <v>143</v>
@@ -3696,10 +3702,10 @@
         <v>88</v>
       </c>
       <c r="C118" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D118" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E118" t="s">
         <v>143</v>
@@ -3730,10 +3736,10 @@
         <v>90</v>
       </c>
       <c r="C120" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D120" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E120" t="s">
         <v>143</v>
@@ -3747,10 +3753,10 @@
         <v>91</v>
       </c>
       <c r="C121" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D121" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E121" t="s">
         <v>143</v>
@@ -3764,10 +3770,10 @@
         <v>92</v>
       </c>
       <c r="C122" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D122" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E122" t="s">
         <v>143</v>
@@ -3781,10 +3787,10 @@
         <v>93</v>
       </c>
       <c r="C123" t="s">
-        <v>185</v>
+        <v>265</v>
       </c>
       <c r="D123" t="s">
-        <v>186</v>
+        <v>266</v>
       </c>
       <c r="E123" t="s">
         <v>143</v>
@@ -3798,10 +3804,10 @@
         <v>94</v>
       </c>
       <c r="C124" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D124" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E124" t="s">
         <v>143</v>
@@ -3815,10 +3821,10 @@
         <v>95</v>
       </c>
       <c r="C125" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D125" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E125" t="s">
         <v>143</v>
@@ -3832,10 +3838,10 @@
         <v>96</v>
       </c>
       <c r="C126" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D126" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E126" t="s">
         <v>143</v>
@@ -3849,10 +3855,10 @@
         <v>97</v>
       </c>
       <c r="C127" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D127" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E127" t="s">
         <v>143</v>
@@ -3866,10 +3872,10 @@
         <v>98</v>
       </c>
       <c r="C128" t="s">
-        <v>187</v>
+        <v>268</v>
       </c>
       <c r="D128" t="s">
-        <v>188</v>
+        <v>267</v>
       </c>
       <c r="E128" t="s">
         <v>143</v>
@@ -3883,10 +3889,10 @@
         <v>99</v>
       </c>
       <c r="C129" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D129" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E129" t="s">
         <v>143</v>
@@ -4223,10 +4229,10 @@
         <v>119</v>
       </c>
       <c r="C149" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D149" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E149" t="s">
         <v>143</v>
@@ -4376,10 +4382,10 @@
         <v>126</v>
       </c>
       <c r="C158" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D158" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E158" t="s">
         <v>143</v>
@@ -4410,10 +4416,10 @@
         <v>128</v>
       </c>
       <c r="C160" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D160" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E160" t="s">
         <v>143</v>
@@ -4444,10 +4450,10 @@
         <v>130</v>
       </c>
       <c r="C162" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D162" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E162" t="s">
         <v>143</v>
@@ -4461,10 +4467,10 @@
         <v>131</v>
       </c>
       <c r="C163" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D163" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E163" t="s">
         <v>143</v>
@@ -4495,10 +4501,10 @@
         <v>133</v>
       </c>
       <c r="C165" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D165" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E165" t="s">
         <v>143</v>
@@ -4512,10 +4518,10 @@
         <v>134</v>
       </c>
       <c r="C166" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D166" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E166" t="s">
         <v>143</v>
@@ -4529,10 +4535,10 @@
         <v>135</v>
       </c>
       <c r="C167" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D167" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E167" t="s">
         <v>143</v>
@@ -4563,10 +4569,10 @@
         <v>137</v>
       </c>
       <c r="C169" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D169" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E169" t="s">
         <v>143</v>
@@ -4597,10 +4603,10 @@
         <v>139</v>
       </c>
       <c r="C171" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D171" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E171" t="s">
         <v>143</v>
@@ -4631,10 +4637,10 @@
         <v>141</v>
       </c>
       <c r="C173" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D173" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E173" t="s">
         <v>143</v>

</xml_diff>